<commit_message>
Files to deal with drugbank.xml, currently store them in a file called drugbank.db
</commit_message>
<xml_diff>
--- a/examples/antibiotics/synthetic_antibiotics_table_realistic.xlsx
+++ b/examples/antibiotics/synthetic_antibiotics_table_realistic.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/examples/antibiotics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2B59D2BFD340584BF941D2F0502B70327747EEAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A05190-2336-7947-8BFD-BEB6266C8384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="95">
   <si>
     <t>note_id</t>
   </si>
@@ -71,9 +71,6 @@
     <t>500 mg</t>
   </si>
   <si>
-    <t>02/11/2023</t>
-  </si>
-  <si>
     <t>note_02</t>
   </si>
   <si>
@@ -83,9 +80,6 @@
     <t>x7 days</t>
   </si>
   <si>
-    <t>09/19/2023</t>
-  </si>
-  <si>
     <t>note_03</t>
   </si>
   <si>
@@ -312,6 +306,18 @@
   </si>
   <si>
     <t>~5 weeks</t>
+  </si>
+  <si>
+    <t>[{"Route": "PO", "Drug Name": "amoxicillin", "Dose": "500 mg", "Frequency": null, "Duration": 3, "Start date": null, "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Route": null, "Drug Name": "Bactrim", "Dose": null, "Frequency": null, "Duration": 7, "Start date": "09/19/2026", "End date": "09/25/2026"}]</t>
+  </si>
+  <si>
+    <t>[{"Route": "PO", "Drug Name": "Azithromycin", "Dose": null, "Frequency": null, "Duration": 5, "Start date": null, "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Route": "PO", "Drug Name": "ciprofloxacin", "Dose": "500 mg", "Frequency": "BID", "Duration": 28, "Start date": null, "End date": null}]</t>
   </si>
 </sst>
 </file>
@@ -347,8 +353,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -651,10 +658,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -680,7 +687,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
@@ -696,59 +703,68 @@
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H2" s="1">
+        <v>44968</v>
+      </c>
+      <c r="K2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>14</v>
       </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H3" s="1">
+        <v>45188</v>
+      </c>
+      <c r="K3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
       </c>
       <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" t="s">
         <v>19</v>
       </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -757,242 +773,245 @@
         <v>11</v>
       </c>
       <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
         <v>24</v>
       </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="K5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
+      <c r="H6" t="s">
         <v>28</v>
       </c>
-      <c r="D6" t="s">
+      <c r="I6" t="s">
         <v>29</v>
       </c>
-      <c r="H6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" t="s">
         <v>32</v>
       </c>
-      <c r="C7" t="s">
+      <c r="I7" t="s">
         <v>33</v>
       </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
         <v>36</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" t="s">
         <v>37</v>
       </c>
-      <c r="E8" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" t="s">
+      <c r="E9" t="s">
         <v>41</v>
       </c>
-      <c r="D9" t="s">
+      <c r="G9" t="s">
         <v>42</v>
       </c>
-      <c r="E9" t="s">
+      <c r="H9" t="s">
         <v>43</v>
       </c>
-      <c r="G9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" t="s">
+      <c r="I11" t="s">
         <v>50</v>
       </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
-      <c r="H11" t="s">
-        <v>51</v>
-      </c>
-      <c r="I11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" t="s">
         <v>53</v>
       </c>
-      <c r="C12" t="s">
+      <c r="F12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" t="s">
         <v>54</v>
       </c>
-      <c r="E12" t="s">
+      <c r="I12" t="s">
         <v>55</v>
       </c>
-      <c r="F12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" t="s">
-        <v>56</v>
-      </c>
-      <c r="I12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" t="s">
         <v>58</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
         <v>59</v>
       </c>
-      <c r="E13" t="s">
+      <c r="G13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" t="s">
         <v>60</v>
       </c>
-      <c r="F13" t="s">
-        <v>61</v>
-      </c>
-      <c r="G13" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" t="s">
         <v>63</v>
       </c>
-      <c r="C14" t="s">
-        <v>64</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" t="s">
         <v>66</v>
       </c>
-      <c r="C15" t="s">
+      <c r="I15" t="s">
         <v>67</v>
       </c>
-      <c r="G15" t="s">
-        <v>68</v>
-      </c>
-      <c r="I15" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" t="s">
         <v>70</v>
       </c>
-      <c r="C16" t="s">
+      <c r="H16" t="s">
         <v>71</v>
       </c>
-      <c r="D16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" t="s">
+      <c r="I16" t="s">
         <v>72</v>
-      </c>
-      <c r="H16" t="s">
-        <v>73</v>
-      </c>
-      <c r="I16" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -1000,19 +1019,19 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s">
         <v>75</v>
       </c>
-      <c r="C17" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" t="s">
-        <v>77</v>
-      </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -1020,22 +1039,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" t="s">
         <v>78</v>
       </c>
-      <c r="C18" t="s">
+      <c r="H18" t="s">
         <v>79</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" t="s">
-        <v>43</v>
-      </c>
-      <c r="F18" t="s">
-        <v>80</v>
-      </c>
-      <c r="H18" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -1043,19 +1062,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" t="s">
         <v>82</v>
       </c>
-      <c r="C19" t="s">
+      <c r="F19" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" t="s">
         <v>83</v>
-      </c>
-      <c r="E19" t="s">
-        <v>84</v>
-      </c>
-      <c r="F19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H19" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
@@ -1063,16 +1082,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" t="s">
         <v>86</v>
-      </c>
-      <c r="C20" t="s">
-        <v>87</v>
-      </c>
-      <c r="D20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -1080,19 +1099,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" t="s">
+        <v>88</v>
+      </c>
+      <c r="E21" t="s">
         <v>89</v>
       </c>
-      <c r="C21" t="s">
+      <c r="F21" t="s">
+        <v>78</v>
+      </c>
+      <c r="G21" t="s">
         <v>90</v>
-      </c>
-      <c r="E21" t="s">
-        <v>91</v>
-      </c>
-      <c r="F21" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New synthetic labels and notes for the new label creation and feature extraction methods that will be commited.
</commit_message>
<xml_diff>
--- a/examples/antibiotics/synthetic_antibiotics_table_realistic.xlsx
+++ b/examples/antibiotics/synthetic_antibiotics_table_realistic.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/examples/antibiotics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A05190-2336-7947-8BFD-BEB6266C8384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8E9B9B-2DD2-1042-9680-649A36777AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1040" windowWidth="30240" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="124">
   <si>
     <t>note_id</t>
   </si>
@@ -308,23 +308,110 @@
     <t>~5 weeks</t>
   </si>
   <si>
-    <t>[{"Route": "PO", "Drug Name": "amoxicillin", "Dose": "500 mg", "Frequency": null, "Duration": 3, "Start date": null, "End date": null}]</t>
-  </si>
-  <si>
-    <t>[{"Route": null, "Drug Name": "Bactrim", "Dose": null, "Frequency": null, "Duration": 7, "Start date": "09/19/2026", "End date": "09/25/2026"}]</t>
-  </si>
-  <si>
-    <t>[{"Route": "PO", "Drug Name": "Azithromycin", "Dose": null, "Frequency": null, "Duration": 5, "Start date": null, "End date": null}]</t>
-  </si>
-  <si>
-    <t>[{"Route": "PO", "Drug Name": "ciprofloxacin", "Dose": "500 mg", "Frequency": "BID", "Duration": 28, "Start date": null, "End date": null}]</t>
+    <t>feature_value</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "amoxicillin", "Route": "PO", "Dose": "500 mg", "Frequency": null, "Duration": 3, "Start date": "02/11/2023", "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "ampicillin-sulbactam", "Route": "IV", "Dose": null, "Frequency": null, "Duration": 5, "Start date": "11/10/2023", "End date": "11/14/2023"}, {"Drug Name": "Augmentin", "Route": null, "Dose": null, "Frequency": null, "Duration": null, "Start date": null, "End date": "11/19/2023"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "Levofloxacin", "Route": null, "Dose": "750 mg", "Frequency": null, "Duration": 5, "Start date": null, "End date": "08/02/2023"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "amoxicillin-clavulanate", "Route": "PO", "Dose": null, "Frequency": "BID", "Duration": 7, "Start date": "06/24/2023", "End date": "06/30/2023"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "azithromycin", "Route": "PO", "Dose": null, "Frequency": null, "Duration": 5, "Start date": "05/01/2024", "End date": "05/05/2024"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "ceftriaxone", "Route": "IM", "Dose": "1g", "Frequency": "once", "Duration": 1, "Start date": "01/13/2024", "End date": "01/13/2024"}, {"Drug Name": "cephalexin", "Route": "PO", "Dose": null, "Frequency": "QID", "Duration": null, "Start date": "01/13/2024", "End date": null}]</t>
+  </si>
+  <si>
+    <t>Extracted multiple drugs, I suppose with the same drug name ?</t>
+  </si>
+  <si>
+    <t>Inferred end date</t>
+  </si>
+  <si>
+    <t>multiple drugs issues</t>
+  </si>
+  <si>
+    <t>Frequency: QID and again multiple drugs</t>
+  </si>
+  <si>
+    <t>another drug with the wrong duration date</t>
+  </si>
+  <si>
+    <t>Translates QID to 4 times a day, Okay solution</t>
+  </si>
+  <si>
+    <t>2nd drug with guessed frequency</t>
+  </si>
+  <si>
+    <t>Took in another drug except the one mentioned</t>
+  </si>
+  <si>
+    <t>Created another drug.Then also guessed the route for the actual drug and missed its dose</t>
+  </si>
+  <si>
+    <t>Guessed the stuff or inferred it idk</t>
+  </si>
+  <si>
+    <t>Completely wrong wtf</t>
+  </si>
+  <si>
+    <t>50% Good labelling</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "trimethoprim-sulfamethoxazole DS", "Route": null, "Dose": null, "Frequency": null, "Duration": 7, "Start date": "09/19/2023", "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "ciprofloxacin", "Route": "PO", "Dose": "500 mg", "Frequency": "BID", "Duration": 28, "Start date": "07/11/2023", "End date": "08/08/2023"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "piperacillin-tazobactam", "Route": "IV", "Dose": null, "Frequency": null, "Duration": 4, "Start date": "02/25/2024", "End date": "02/28/2024"}, {"Drug Name": "cipro", "Route": "PO", "Dose": null, "Frequency": null, "Duration": 7, "Start date": "02/28/2024", "End date": "03/06/2024"}, {"Drug Name": "Flagyl", "Route": "PO", "Dose": null, "Frequency": null, "Duration": 7, "Start date": "02/28/2024", "End date": "03/06/2024"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "vancomycin", "Route": "IV", "Dose": "NULL", "Frequency": "NULL", "Duration": 5, "Start date": "09/17/2022", "End date": "09/22/2022"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "doxycycline", "Route": "NULL", "Dose": "100 mg", "Frequency": "BID", "Duration": 21, "Start date": "NULL", "End date": "09/14/2023"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "clindamycin", "Route": null, "Dose": "300 mg", "Frequency": "QID", "Duration": 7, "Start date": null, "End date": "04/21/2024"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "cefazolin", "Route": "IV", "Dose": null, "Frequency": null, "Duration": null, "Start date": "10/22/2023", "End date": null}, {"Drug Name": "cephalexin", "Route": "PO", "Dose": null, "Frequency": "QID", "Duration": 2, "Start date": null, "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "nitrofurantoin", "Route": null, "Dose": null, "Frequency": null, "Duration": 5, "Start date": null, "End date": "07/08/2024"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "Meropenem", "Route": "IV", "Dose": "NULL", "Frequency": "NULL", "Duration": 14, "Start date": "11/12/2023", "End date": "11/25/2023"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "acyclovir", "Route": null, "Dose": "400 mg", "Frequency": "BID", "Duration": null, "Start date": null, "End date": null}, {"Drug Name": "fluconazole", "Route": null, "Dose": "400 mg", "Frequency": "daily", "Duration": null, "Start date": null, "End date": null}, {"Drug Name": "levofloxacin", "Route": null, "Dose": "500 mg", "Frequency": "daily", "Duration": null, "Start date": null, "End date": null}, {"Drug Name": "cefepime", "Route": "IV", "Dose": "2 g", "Frequency": null, "Duration": 5, "Start date": null, "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "ertapenem", "Route": "IV", "Dose": "1g", "Frequency": "daily", "Duration": 21, "Start date": "04/25/2024", "End date": "05/15/2024"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "Vancomycin", "Route": "IV", "Dose": null, "Frequency": null, "Duration": 3, "Start date": null, "End date": null}, {"Drug Name": "Linezolid", "Route": null, "Dose": "600 mg", "Frequency": "BID", "Duration": 20, "Start date": "01/31/2024", "End date": null}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "daptomycin", "Route": "IV", "Dose": "8 mg/kg", "Frequency": "NULL", "Duration": 42, "Start date": "NULL", "End date": "NULL"}]</t>
+  </si>
+  <si>
+    <t>[{"Drug Name": "Fluconazole", "Route": "NULL", "Dose": "400 mg", "Frequency": "daily", "Duration": 35, "Start date": "NULL", "End date": "NULL"}, {"Drug Name": "Acyclovir", "Route": "NULL", "Dose": "400 mg", "Frequency": "BID", "Duration": "NULL", "Start date": "NULL", "End date": "NULL"}, {"Drug Name": "TMP-SMX", "Route": "NULL", "Dose": "NULL", "Frequency": "three times per week", "Duration": "NULL", "Start date": "NULL", "End date": "NULL"}]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -332,13 +419,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -350,14 +457,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="40% - Accent2" xfId="1" builtinId="35"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -658,463 +780,800 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Z22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="18" max="18" width="8.83203125" style="3"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5"/>
+    </row>
+    <row r="2" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="1">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="2">
         <v>44968</v>
       </c>
-      <c r="K2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I2" s="1"/>
+      <c r="J2" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="6"/>
+    </row>
+    <row r="3" spans="1:26" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45188</v>
       </c>
-      <c r="K3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I3" s="1"/>
+      <c r="J3" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="6"/>
+      <c r="S3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G4" t="s">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J4" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="4"/>
+    </row>
+    <row r="5" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I5" s="1"/>
+      <c r="J5" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H6" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H7" t="s">
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J7" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E8" t="s">
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G8" t="s">
+      <c r="F8" s="1"/>
+      <c r="G8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I8" t="s">
+      <c r="H8" s="1"/>
+      <c r="I8" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+    </row>
+    <row r="9" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>38</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G9" t="s">
+      <c r="F9" s="1"/>
+      <c r="G9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I9" s="1"/>
+      <c r="J9" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>44</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F10" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I10" s="1"/>
+      <c r="J10" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+    </row>
+    <row r="11" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>47</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H11" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J11" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>51</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E12" t="s">
+      <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I12" t="s">
+      <c r="H12" s="1"/>
+      <c r="I12" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J12" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+    </row>
+    <row r="13" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>56</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E13" t="s">
+      <c r="D13" s="1"/>
+      <c r="E13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I13" t="s">
+      <c r="H13" s="1"/>
+      <c r="I13" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J13" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>61</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H14" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I14" s="1"/>
+      <c r="J14" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>64</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G15" t="s">
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="I15" t="s">
+      <c r="H15" s="1"/>
+      <c r="I15" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J15" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+    </row>
+    <row r="16" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>68</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G16" t="s">
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="J16" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+    </row>
+    <row r="17" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>73</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G17" t="s">
+      <c r="F17" s="1"/>
+      <c r="G17" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>76</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H18" t="s">
+      <c r="G18" s="1"/>
+      <c r="H18" s="1" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I18" s="1"/>
+      <c r="J18" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+    </row>
+    <row r="19" spans="1:18" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>80</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E19" t="s">
+      <c r="D19" s="1"/>
+      <c r="E19" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H19" t="s">
+      <c r="G19" s="1"/>
+      <c r="H19" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="1"/>
+      <c r="J19" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>84</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>87</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E21" t="s">
+      <c r="D21" s="1"/>
+      <c r="E21" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
     </row>
   </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="J21:Q21"/>
+    <mergeCell ref="J22:Q22"/>
+    <mergeCell ref="J16:Q16"/>
+    <mergeCell ref="J17:Q17"/>
+    <mergeCell ref="J18:Q18"/>
+    <mergeCell ref="J19:Q19"/>
+    <mergeCell ref="J20:Q20"/>
+    <mergeCell ref="J11:Q11"/>
+    <mergeCell ref="J12:Q12"/>
+    <mergeCell ref="J13:Q13"/>
+    <mergeCell ref="J14:Q14"/>
+    <mergeCell ref="J15:Q15"/>
+    <mergeCell ref="J2:Q2"/>
+    <mergeCell ref="J3:Q3"/>
+    <mergeCell ref="J4:Q4"/>
+    <mergeCell ref="J5:Q5"/>
+    <mergeCell ref="J6:Q6"/>
+    <mergeCell ref="J7:Q7"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="T1:Z1"/>
+    <mergeCell ref="J1:Q1"/>
+    <mergeCell ref="J9:Q9"/>
+    <mergeCell ref="J10:Q10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>